<commit_message>
Port framework to Thinking-Tester Contact List
Migrate the test framework and tests from the Saucedemo sample to the Thinking-Tester Contact List app. Updates include: switch config/test URLs to the contact-list app and add credentials; remove old saucedemo-specific page objects and tests; add new page objects for contact flows (Add/Edit/Details/List, SignUp, Login); refactor BasePage (rename methods, add visibility, select/hover/alert helpers, improved waits and logging); enhance test infra (base_test and conftest) with multi-browser support, worker-scoped logging, improved screenshot handling and Allure attachments; add run_tests helper, update setup_framework, add new test files and test data, and update requirements. This change prepares the suite for the new application under test and improves robustness of browser and logging utilities.
</commit_message>
<xml_diff>
--- a/test_data/TestData_AppName.xlsx
+++ b/test_data/TestData_AppName.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\TY_New\PythonRMG\HarshaFW_Python\test_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\PycharmProjects\Python_Selenium_FW_PY07\test_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DBB6BAD-A539-478D-A81B-3876314C6D6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15460" windowHeight="5160" firstSheet="1" activeTab="3"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Module_Flow" sheetId="61" r:id="rId1"/>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="21">
   <si>
     <t>PRODUCT_NAME</t>
   </si>
@@ -64,42 +65,6 @@
   </si>
   <si>
     <t>Module_Name</t>
-  </si>
-  <si>
-    <t>SALUTATION</t>
-  </si>
-  <si>
-    <t>FIRST_NAME</t>
-  </si>
-  <si>
-    <t>LAST_NAME</t>
-  </si>
-  <si>
-    <t>PR_AGE</t>
-  </si>
-  <si>
-    <t>RESIDENTAIL_STATE</t>
-  </si>
-  <si>
-    <t>PLANED_RETIREMENT_AGE</t>
-  </si>
-  <si>
-    <t>ANNUAL_INCOME</t>
-  </si>
-  <si>
-    <t>Mr</t>
-  </si>
-  <si>
-    <t>ANDHRA PRADESH</t>
-  </si>
-  <si>
-    <t>60</t>
-  </si>
-  <si>
-    <t>Harsha</t>
-  </si>
-  <si>
-    <t>K B</t>
   </si>
   <si>
     <t>GAURANTEEDASSUREDINCOME</t>
@@ -126,7 +91,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="15">
     <font>
       <sz val="11"/>
@@ -232,7 +197,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -242,6 +207,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -319,62 +290,64 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="9">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+  <cellXfs count="11">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="39" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="39" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="39" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="39" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="40">
-    <cellStyle name="Hyperlink 2" xfId="4"/>
-    <cellStyle name="Hyperlink 3" xfId="6"/>
-    <cellStyle name="Hyperlink 4" xfId="8"/>
+    <cellStyle name="Hyperlink 2" xfId="4" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
+    <cellStyle name="Hyperlink 3" xfId="6" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="Hyperlink 4" xfId="8" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 10" xfId="17"/>
-    <cellStyle name="Normal 11" xfId="18"/>
-    <cellStyle name="Normal 12" xfId="20"/>
-    <cellStyle name="Normal 13" xfId="21"/>
-    <cellStyle name="Normal 14" xfId="29"/>
-    <cellStyle name="Normal 15" xfId="38"/>
-    <cellStyle name="Normal 16" xfId="30"/>
-    <cellStyle name="Normal 17" xfId="39"/>
-    <cellStyle name="Normal 2" xfId="1"/>
-    <cellStyle name="Normal 3" xfId="3"/>
-    <cellStyle name="Normal 4" xfId="5"/>
-    <cellStyle name="Normal 5" xfId="7"/>
-    <cellStyle name="Normal 5 2" xfId="11"/>
-    <cellStyle name="Normal 5 2 2" xfId="14"/>
-    <cellStyle name="Normal 5 2 2 2" xfId="26"/>
-    <cellStyle name="Normal 5 2 2 3" xfId="35"/>
-    <cellStyle name="Normal 5 2 3" xfId="23"/>
-    <cellStyle name="Normal 5 2 4" xfId="32"/>
-    <cellStyle name="Normal 5 3" xfId="13"/>
-    <cellStyle name="Normal 5 3 2" xfId="25"/>
-    <cellStyle name="Normal 5 3 3" xfId="34"/>
-    <cellStyle name="Normal 5 4" xfId="16"/>
-    <cellStyle name="Normal 5 4 2" xfId="27"/>
-    <cellStyle name="Normal 5 4 3" xfId="36"/>
-    <cellStyle name="Normal 5 5" xfId="19"/>
-    <cellStyle name="Normal 5 5 2" xfId="28"/>
-    <cellStyle name="Normal 5 5 3" xfId="37"/>
-    <cellStyle name="Normal 5 6" xfId="22"/>
-    <cellStyle name="Normal 5 7" xfId="31"/>
-    <cellStyle name="Normal 6" xfId="9"/>
-    <cellStyle name="Normal 7" xfId="10"/>
-    <cellStyle name="Normal 8" xfId="12"/>
-    <cellStyle name="Normal 8 2" xfId="24"/>
-    <cellStyle name="Normal 8 3" xfId="33"/>
-    <cellStyle name="Normal 9" xfId="15"/>
-    <cellStyle name="Percent 2" xfId="2"/>
+    <cellStyle name="Normal 10" xfId="17" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
+    <cellStyle name="Normal 11" xfId="18" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
+    <cellStyle name="Normal 12" xfId="20" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
+    <cellStyle name="Normal 13" xfId="21" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
+    <cellStyle name="Normal 14" xfId="29" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
+    <cellStyle name="Normal 15" xfId="38" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
+    <cellStyle name="Normal 16" xfId="30" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
+    <cellStyle name="Normal 17" xfId="39" xr:uid="{00000000-0005-0000-0000-00000B000000}"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-00000C000000}"/>
+    <cellStyle name="Normal 3" xfId="3" xr:uid="{00000000-0005-0000-0000-00000D000000}"/>
+    <cellStyle name="Normal 4" xfId="5" xr:uid="{00000000-0005-0000-0000-00000E000000}"/>
+    <cellStyle name="Normal 5" xfId="7" xr:uid="{00000000-0005-0000-0000-00000F000000}"/>
+    <cellStyle name="Normal 5 2" xfId="11" xr:uid="{00000000-0005-0000-0000-000010000000}"/>
+    <cellStyle name="Normal 5 2 2" xfId="14" xr:uid="{00000000-0005-0000-0000-000011000000}"/>
+    <cellStyle name="Normal 5 2 2 2" xfId="26" xr:uid="{00000000-0005-0000-0000-000012000000}"/>
+    <cellStyle name="Normal 5 2 2 3" xfId="35" xr:uid="{00000000-0005-0000-0000-000013000000}"/>
+    <cellStyle name="Normal 5 2 3" xfId="23" xr:uid="{00000000-0005-0000-0000-000014000000}"/>
+    <cellStyle name="Normal 5 2 4" xfId="32" xr:uid="{00000000-0005-0000-0000-000015000000}"/>
+    <cellStyle name="Normal 5 3" xfId="13" xr:uid="{00000000-0005-0000-0000-000016000000}"/>
+    <cellStyle name="Normal 5 3 2" xfId="25" xr:uid="{00000000-0005-0000-0000-000017000000}"/>
+    <cellStyle name="Normal 5 3 3" xfId="34" xr:uid="{00000000-0005-0000-0000-000018000000}"/>
+    <cellStyle name="Normal 5 4" xfId="16" xr:uid="{00000000-0005-0000-0000-000019000000}"/>
+    <cellStyle name="Normal 5 4 2" xfId="27" xr:uid="{00000000-0005-0000-0000-00001A000000}"/>
+    <cellStyle name="Normal 5 4 3" xfId="36" xr:uid="{00000000-0005-0000-0000-00001B000000}"/>
+    <cellStyle name="Normal 5 5" xfId="19" xr:uid="{00000000-0005-0000-0000-00001C000000}"/>
+    <cellStyle name="Normal 5 5 2" xfId="28" xr:uid="{00000000-0005-0000-0000-00001D000000}"/>
+    <cellStyle name="Normal 5 5 3" xfId="37" xr:uid="{00000000-0005-0000-0000-00001E000000}"/>
+    <cellStyle name="Normal 5 6" xfId="22" xr:uid="{00000000-0005-0000-0000-00001F000000}"/>
+    <cellStyle name="Normal 5 7" xfId="31" xr:uid="{00000000-0005-0000-0000-000020000000}"/>
+    <cellStyle name="Normal 6" xfId="9" xr:uid="{00000000-0005-0000-0000-000021000000}"/>
+    <cellStyle name="Normal 7" xfId="10" xr:uid="{00000000-0005-0000-0000-000022000000}"/>
+    <cellStyle name="Normal 8" xfId="12" xr:uid="{00000000-0005-0000-0000-000023000000}"/>
+    <cellStyle name="Normal 8 2" xfId="24" xr:uid="{00000000-0005-0000-0000-000024000000}"/>
+    <cellStyle name="Normal 8 3" xfId="33" xr:uid="{00000000-0005-0000-0000-000025000000}"/>
+    <cellStyle name="Normal 9" xfId="15" xr:uid="{00000000-0005-0000-0000-000026000000}"/>
+    <cellStyle name="Percent 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000027000000}"/>
   </cellStyles>
   <dxfs count="1">
     <dxf>
@@ -597,15 +570,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="36.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.4140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="36.19921875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="14.5">
+    <row r="1" spans="1:2" ht="14.4">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -613,7 +586,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="14.5">
+    <row r="2" spans="1:2" ht="14.4">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -621,7 +594,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="14.5">
+    <row r="3" spans="1:2" ht="14.4">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -629,7 +602,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="14.5">
+    <row r="4" spans="1:2" ht="14.4">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
@@ -643,17 +616,17 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="36.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.75" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.4140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="36.19921875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.69921875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.3984375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="14.5">
+    <row r="1" spans="1:4" ht="14.4">
       <c r="A1" s="5" t="s">
         <v>13</v>
       </c>
@@ -667,9 +640,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="14.5">
+    <row r="2" spans="1:4" ht="14.4">
       <c r="A2" s="1" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>8</v>
@@ -681,9 +654,9 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="14.5">
+    <row r="3" spans="1:4" ht="14.4">
       <c r="A3" s="1" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>11</v>
@@ -695,9 +668,9 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="14.5">
+    <row r="4" spans="1:4" ht="14.4">
       <c r="A4" s="1" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>12</v>
@@ -711,7 +684,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C4">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C4" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -720,36 +693,36 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="24.6640625" customWidth="1" collapsed="1"/>
-    <col min="2" max="2" width="15.08203125" customWidth="1" collapsed="1"/>
+    <col min="1" max="1" width="24.69921875" customWidth="1" collapsed="1"/>
+    <col min="2" max="2" width="15.09765625" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="14.5">
+    <row r="1" spans="1:2" ht="14.4">
       <c r="A1" s="4" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" ht="14.5">
-      <c r="A2" s="8" t="s">
-        <v>30</v>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="14.4">
+      <c r="A2" s="6" t="s">
+        <v>18</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="14.5">
-      <c r="A3" s="8" t="s">
-        <v>31</v>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="14.4">
+      <c r="A3" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -759,97 +732,63 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:I4"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="10.75" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.4140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.69921875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.3984375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.83203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.25" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.9140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.58203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.19921875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.8984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="14.5">
-      <c r="A1" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="F1" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="G1" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="H1" s="7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8">
-      <c r="A2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E2" s="2">
-        <v>37</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="H2" s="2">
-        <v>1000000</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8">
-      <c r="A3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E3" s="2">
-        <v>31</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="H3" s="2">
-        <v>1000000</v>
-      </c>
+    <row r="1" spans="1:9" ht="14.4">
+      <c r="A1" s="7"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="8"/>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" s="9"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="8"/>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" s="9"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="8"/>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" s="8"/>
+      <c r="B4" s="8"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="8"/>
+      <c r="I4" s="8"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:H1">

</xml_diff>